<commit_message>
feat: CLI con --dry-run, --rejects, --report y --force
- cli: entradas por archivo o carpeta, -c/-o, --rejects (datos originales sin
  enmascarar, avisado en --help y en consola), --report JSON enmascarado,
  --dry-run sin crear archivos ni carpetas, --force para sobrescribir.
- Errores en español sin traza: 1 entrada/config/escritura, 2 argumentos.
- readers/config convierten errores de lectura en ReaderError/ConfigError.
- Generador: caso de fusión dudosa (dos personas comparten teléfono);
  esperados 68 leídas, 21 duplicados, 44 en salida, 1 fusión dudosa.
- README: uso, opciones y aviso sobre --rejects.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/input/eventos.xlsx
+++ b/examples/input/eventos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1021,6 +1021,31 @@
         <v>45921</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Héctor</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gallardo Rey</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>600000758</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>hector.g@example.org</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>45870</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>